<commit_message>
Tier 1 valuation fixes: dated DCF, funded terminal value, APSEZ live model
- DCF discounts from the net-debt date with a first-year stub and rolls
  equity to the cover date (JSW counted Q1 FY27 twice before).
- Terminal value uses the value-driver formula at RONIC = own FY24-26 ROIC
  (JSW 12.0%, APSEZ 10.5%) instead of Gordon on final-year FCFF.
- JSW: target 170 -> 185, SELL; perpetuity 121 (bull 129, bear 58).
- APSEZ: three-statement DCF, live-formula Excel, data-driven prose and
  charts; target 1,165 -> 1,195; REDUCE -> SELL under the house policy.
- selftest.py: syntax, regression, three-statement rebuild, LibreOffice
  workbook check, packaging and copy sync. Tab indentation removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/JSWINFRA/JSW_Infrastructure_Ltd_ERIP_Model.xlsx
+++ b/reports/JSWINFRA/JSW_Infrastructure_Ltd_ERIP_Model.xlsx
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="549" uniqueCount="318">
   <si>
     <t xml:space="preserve">JSW Infrastructure Ltd - three-statement model</t>
   </si>
@@ -765,7 +765,7 @@
     <t xml:space="preserve">JSW Infrastructure Ltd - DCF</t>
   </si>
   <si>
-    <t xml:space="preserve">FCFF from the linked statements; mid-year discounting; Gordon terminal value; exit-multiple target</t>
+    <t xml:space="preserve">FCFF from the linked statements; stub-period discounting from the balance-sheet date; exit-multiple target</t>
   </si>
   <si>
     <t xml:space="preserve">    NOPAT  (EBIT x (1 - tax rate))</t>
@@ -780,10 +780,28 @@
     <t xml:space="preserve">    Less: increase in net operating assets</t>
   </si>
   <si>
-    <t xml:space="preserve">Discounting</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    Discount period (mid-year)</t>
+    <t xml:space="preserve">Timing and discounting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Balance-sheet date (date of the net debt)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash flows before it are inside net debt</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    First forecast year ends</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Valuation date (cover)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Share of the first year counted (stub)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Share of year counted</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Discount period (years from balance-sheet date, mid-year)</t>
   </si>
   <si>
     <t xml:space="preserve">    Discount factor</t>
@@ -792,19 +810,28 @@
     <t xml:space="preserve">    Present value of FCFF</t>
   </si>
   <si>
-    <t xml:space="preserve">Valuation: perpetuity growth</t>
+    <t xml:space="preserve">Valuation: perpetuity</t>
   </si>
   <si>
     <t xml:space="preserve">    WACC</t>
   </si>
   <si>
+    <t xml:space="preserve">    Return on new invested capital in perpetuity (RONIC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assumptions.json terminal_ronic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Terminal reinvestment rate  (g / RONIC, share of NOPAT)</t>
+  </si>
+  <si>
     <t xml:space="preserve">    Sum of PV of FCFF</t>
   </si>
   <si>
-    <t xml:space="preserve">    Terminal value  (FCFF N x (1 + g) / (WACC - g))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    PV of terminal value  (discounted at N - 0.5)</t>
+    <t xml:space="preserve">    Terminal value  (NOPAT N x (1 + g) x (1 - g / RONIC) / (WACC - g))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    PV of terminal value  (at the final cash flow's period)</t>
   </si>
   <si>
     <t xml:space="preserve">Enterprise value</t>
@@ -813,10 +840,10 @@
     <t xml:space="preserve">    Terminal value as % of EV</t>
   </si>
   <si>
-    <t xml:space="preserve">    Net debt  (negative = net cash)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Net debt at the valuation date (assumptions.json)</t>
+    <t xml:space="preserve">    Net debt at the balance-sheet date  (negative = net cash)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">assumptions.json net_debt, as at the balance-sheet date</t>
   </si>
   <si>
     <t xml:space="preserve">    Non-operating assets</t>
@@ -825,7 +852,16 @@
     <t xml:space="preserve">Treasury investments and stakes not in FCFF</t>
   </si>
   <si>
-    <t xml:space="preserve">Equity value</t>
+    <t xml:space="preserve">    Equity value at the balance-sheet date</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Cost of equity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">    Roll-forward to the valuation date  ((1 + ke) ^ years)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equity value at the valuation date</t>
   </si>
   <si>
     <t xml:space="preserve">    Shares outstanding (Cr)</t>
@@ -955,7 +991,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="16">
+  <numFmts count="17">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0;\(#,##0.0\);\-"/>
     <numFmt numFmtId="166" formatCode="0.0%;\(0.0%\)"/>
@@ -969,9 +1005,10 @@
     <numFmt numFmtId="174" formatCode="#,##0.000;\(#,##0.000\)"/>
     <numFmt numFmtId="175" formatCode="0.00"/>
     <numFmt numFmtId="176" formatCode="0.00%"/>
-    <numFmt numFmtId="177" formatCode="0.0"/>
+    <numFmt numFmtId="177" formatCode="dd\-mmm\-yyyy"/>
     <numFmt numFmtId="178" formatCode="0.000"/>
-    <numFmt numFmtId="179" formatCode="0.0\x"/>
+    <numFmt numFmtId="179" formatCode="0.0000"/>
+    <numFmt numFmtId="180" formatCode="0.0\x"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -1228,7 +1265,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="79">
+  <cellXfs count="80">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1505,11 +1542,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="178" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="178" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1521,6 +1558,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="175" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1529,15 +1570,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="180" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="180" fontId="18" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="179" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="180" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2254,10 +2295,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K52"/>
+  <dimension ref="A1:K62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="2" style="0" width="11"/>
   </cols>
   <sheetData>
@@ -2726,367 +2767,394 @@
         <v>250</v>
       </c>
       <c r="B17" s="68" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C17" s="69" t="n">
-        <f aca="false">B17+1</f>
-        <v>1.5</v>
-      </c>
-      <c r="D17" s="69" t="n">
-        <f aca="false">C17+1</f>
-        <v>2.5</v>
-      </c>
-      <c r="E17" s="69" t="n">
-        <f aca="false">D17+1</f>
-        <v>3.5</v>
-      </c>
-      <c r="F17" s="69" t="n">
-        <f aca="false">E17+1</f>
-        <v>4.5</v>
-      </c>
-      <c r="G17" s="69" t="n">
-        <f aca="false">F17+1</f>
-        <v>5.5</v>
-      </c>
-      <c r="H17" s="69" t="n">
-        <f aca="false">G17+1</f>
-        <v>6.5</v>
-      </c>
-      <c r="I17" s="69" t="n">
-        <f aca="false">H17+1</f>
-        <v>7.5</v>
-      </c>
-      <c r="J17" s="69" t="n">
-        <f aca="false">I17+1</f>
-        <v>8.5</v>
-      </c>
-      <c r="K17" s="69" t="n">
-        <f aca="false">J17+1</f>
-        <v>9.5</v>
+        <v>46203</v>
+      </c>
+      <c r="C17" s="62" t="s">
+        <v>251</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="B18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^B17</f>
-        <v>0.946998061410397</v>
-      </c>
-      <c r="C18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^C17</f>
-        <v>0.849272907376867</v>
-      </c>
-      <c r="D18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^D17</f>
-        <v>0.761632468529188</v>
-      </c>
-      <c r="E18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^E17</f>
-        <v>0.68303605599472</v>
-      </c>
-      <c r="F18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^F17</f>
-        <v>0.612550374447362</v>
-      </c>
-      <c r="G18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^G17</f>
-        <v>0.549338439665773</v>
-      </c>
-      <c r="H18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^H17</f>
-        <v>0.492649639740541</v>
-      </c>
-      <c r="I18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^I17</f>
-        <v>0.441810821911807</v>
-      </c>
-      <c r="J18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^J17</f>
-        <v>0.39621829919776</v>
-      </c>
-      <c r="K18" s="70" t="n">
-        <f aca="false">1/(1+WACC!$B$18)^K17</f>
-        <v>0.355330681896478</v>
+        <v>252</v>
+      </c>
+      <c r="B18" s="68" t="n">
+        <v>46477</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="B19" s="43" t="n">
-        <f aca="false">B14*B18</f>
-        <v>-4835.67530886638</v>
-      </c>
-      <c r="C19" s="43" t="n">
-        <f aca="false">C14*C18</f>
-        <v>-4396.78878926336</v>
-      </c>
-      <c r="D19" s="43" t="n">
-        <f aca="false">D14*D18</f>
-        <v>565.83948343072</v>
-      </c>
-      <c r="E19" s="43" t="n">
-        <f aca="false">E14*E18</f>
-        <v>1999.51636839124</v>
-      </c>
-      <c r="F19" s="43" t="n">
-        <f aca="false">F14*F18</f>
-        <v>2202.98404502115</v>
-      </c>
-      <c r="G19" s="43" t="n">
-        <f aca="false">G14*G18</f>
-        <v>2083.05312635143</v>
-      </c>
-      <c r="H19" s="43" t="n">
-        <f aca="false">H14*H18</f>
-        <v>1948.23716355807</v>
-      </c>
-      <c r="I19" s="43" t="n">
-        <f aca="false">I14*I18</f>
-        <v>1838.2121663441</v>
-      </c>
-      <c r="J19" s="43" t="n">
-        <f aca="false">J14*J18</f>
-        <v>1729.59648378028</v>
-      </c>
-      <c r="K19" s="43" t="n">
-        <f aca="false">K14*K18</f>
-        <v>1626.69967043695</v>
+        <v>253</v>
+      </c>
+      <c r="B19" s="68" t="n">
+        <v>46296</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="B20" s="69" t="n">
+        <f aca="false">MIN(1,MAX(0,(B18-B17)/365.25))</f>
+        <v>0.750171115674196</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="30" t="s">
-        <v>253</v>
+      <c r="A21" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B21" s="69" t="n">
+        <f aca="false">$B$20</f>
+        <v>0.750171115674196</v>
+      </c>
+      <c r="C21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" s="70" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>254</v>
-      </c>
-      <c r="B22" s="71" t="n">
+        <v>256</v>
+      </c>
+      <c r="B22" s="64" t="n">
+        <f aca="false">$B$20*0.5</f>
+        <v>0.375085557837098</v>
+      </c>
+      <c r="C22" s="64" t="n">
+        <f aca="false">$B$20+0.5</f>
+        <v>1.2501711156742</v>
+      </c>
+      <c r="D22" s="64" t="n">
+        <f aca="false">C22+1</f>
+        <v>2.2501711156742</v>
+      </c>
+      <c r="E22" s="64" t="n">
+        <f aca="false">D22+1</f>
+        <v>3.2501711156742</v>
+      </c>
+      <c r="F22" s="64" t="n">
+        <f aca="false">E22+1</f>
+        <v>4.2501711156742</v>
+      </c>
+      <c r="G22" s="64" t="n">
+        <f aca="false">F22+1</f>
+        <v>5.2501711156742</v>
+      </c>
+      <c r="H22" s="64" t="n">
+        <f aca="false">G22+1</f>
+        <v>6.2501711156742</v>
+      </c>
+      <c r="I22" s="64" t="n">
+        <f aca="false">H22+1</f>
+        <v>7.2501711156742</v>
+      </c>
+      <c r="J22" s="64" t="n">
+        <f aca="false">I22+1</f>
+        <v>8.2501711156742</v>
+      </c>
+      <c r="K22" s="64" t="n">
+        <f aca="false">J22+1</f>
+        <v>9.2501711156742</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="B23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^B22</f>
+        <v>0.959970241613785</v>
+      </c>
+      <c r="C23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^C22</f>
+        <v>0.87269930645706</v>
+      </c>
+      <c r="D23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^D22</f>
+        <v>0.78264138804754</v>
+      </c>
+      <c r="E23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^E22</f>
+        <v>0.70187696696092</v>
+      </c>
+      <c r="F23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^F22</f>
+        <v>0.629447003792159</v>
+      </c>
+      <c r="G23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^G22</f>
+        <v>0.564491426892752</v>
+      </c>
+      <c r="H23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^H22</f>
+        <v>0.506238919425585</v>
+      </c>
+      <c r="I23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^I22</f>
+        <v>0.453997760341318</v>
+      </c>
+      <c r="J23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^J22</f>
+        <v>0.407147610517193</v>
+      </c>
+      <c r="K23" s="69" t="n">
+        <f aca="false">1/(1+WACC!$B$18)^K22</f>
+        <v>0.365132146522559</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="B24" s="43" t="n">
+        <f aca="false">B14*B21*B23</f>
+        <v>-3677.2753553481</v>
+      </c>
+      <c r="C24" s="43" t="n">
+        <f aca="false">C14*C21*C23</f>
+        <v>-4518.07009701959</v>
+      </c>
+      <c r="D24" s="43" t="n">
+        <f aca="false">D14*D21*D23</f>
+        <v>581.447636521486</v>
+      </c>
+      <c r="E24" s="43" t="n">
+        <f aca="false">E14*E21*E23</f>
+        <v>2054.67115786638</v>
+      </c>
+      <c r="F24" s="43" t="n">
+        <f aca="false">F14*F21*F23</f>
+        <v>2263.75130011394</v>
+      </c>
+      <c r="G24" s="43" t="n">
+        <f aca="false">G14*G21*G23</f>
+        <v>2140.51219918807</v>
+      </c>
+      <c r="H24" s="43" t="n">
+        <f aca="false">H14*H21*H23</f>
+        <v>2001.97746411392</v>
+      </c>
+      <c r="I24" s="43" t="n">
+        <f aca="false">I14*I21*I23</f>
+        <v>1888.91753022512</v>
+      </c>
+      <c r="J24" s="43" t="n">
+        <f aca="false">J14*J21*J23</f>
+        <v>1777.3057856134</v>
+      </c>
+      <c r="K24" s="43" t="n">
+        <f aca="false">K14*K21*K23</f>
+        <v>1671.57065988248</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="30" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
+        <v>260</v>
+      </c>
+      <c r="B27" s="71" t="n">
         <f aca="false">WACC!$B$18</f>
         <v>0.1150692</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="B23" s="18" t="n">
+      <c r="B28" s="18" t="n">
         <f aca="false">Scenarios!$B$39</f>
         <v>0.04</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>255</v>
-      </c>
-      <c r="B24" s="43" t="n">
-        <f aca="false">SUM(B19:K19)</f>
-        <v>4761.67440918421</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>256</v>
-      </c>
-      <c r="B25" s="43" t="n">
-        <f aca="false">K14*(1+B23)/(B22-B23)</f>
-        <v>63422.9182238854</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>257</v>
-      </c>
-      <c r="B26" s="43" t="n">
-        <f aca="false">B25/(1+B22)^K17</f>
-        <v>22536.1087803578</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="2" t="s">
-        <v>258</v>
-      </c>
-      <c r="B27" s="54" t="n">
-        <f aca="false">B24+B26</f>
-        <v>27297.783189542</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
-        <v>259</v>
-      </c>
-      <c r="B28" s="34" t="n">
-        <f aca="false">B26/B27</f>
-        <v>0.82556552756971</v>
-      </c>
-    </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>260</v>
-      </c>
-      <c r="B29" s="72" t="n">
-        <v>-2769</v>
+        <v>261</v>
+      </c>
+      <c r="B29" s="31" t="n">
+        <v>0.12</v>
       </c>
       <c r="C29" s="62" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>262</v>
-      </c>
-      <c r="B30" s="72" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="62" t="s">
         <v>263</v>
       </c>
+      <c r="B30" s="34" t="n">
+        <f aca="false">$B$28/$B$29</f>
+        <v>0.333333333333333</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2" t="s">
+      <c r="A31" s="3" t="s">
         <v>264</v>
       </c>
-      <c r="B31" s="54" t="n">
-        <f aca="false">B27-B29+B30</f>
-        <v>30066.783189542</v>
+      <c r="B31" s="43" t="n">
+        <f aca="false">SUM(B24:K24)</f>
+        <v>6184.80828115711</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
         <v>265</v>
       </c>
-      <c r="B32" s="73" t="n">
+      <c r="B32" s="43" t="n">
+        <f aca="false">K10*(1+$B$28)*(1-$B$28/$B$29)/($B$27-$B$28)</f>
+        <v>50281.0283946773</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="B33" s="43" t="n">
+        <f aca="false">$B$32/(1+$B$27)^K22</f>
+        <v>18359.2198271103</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="2" t="s">
+        <v>267</v>
+      </c>
+      <c r="B34" s="54" t="n">
+        <f aca="false">$B$31+$B$33</f>
+        <v>24544.0281082674</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="B35" s="34" t="n">
+        <f aca="false">$B$33/$B$34</f>
+        <v>0.748011685210146</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>269</v>
+      </c>
+      <c r="B36" s="72" t="n">
+        <v>-2769</v>
+      </c>
+      <c r="C36" s="62" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>271</v>
+      </c>
+      <c r="B37" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="C37" s="62" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B38" s="43" t="n">
+        <f aca="false">$B$34-$B$36+$B$37</f>
+        <v>27313.0281082674</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="3" t="s">
+        <v>274</v>
+      </c>
+      <c r="B39" s="18" t="n">
+        <f aca="false">WACC!$B$10</f>
+        <v>0.123315</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
+        <v>275</v>
+      </c>
+      <c r="B40" s="73" t="n">
+        <f aca="false">(1+$B$39)^((B19-B17)/365.25)</f>
+        <v>1.03005096417884</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="2" t="s">
+        <v>276</v>
+      </c>
+      <c r="B41" s="54" t="n">
+        <f aca="false">$B$38*$B$40</f>
+        <v>28133.8109375647</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="3" t="s">
+        <v>277</v>
+      </c>
+      <c r="B42" s="74" t="n">
         <f aca="false">Schedules!K23</f>
         <v>232.35</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="2" t="s">
-        <v>266</v>
-      </c>
-      <c r="B33" s="38" t="n">
-        <f aca="false">B31/B32</f>
-        <v>129.40298338516</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="3" t="s">
-        <v>267</v>
-      </c>
-      <c r="B34" s="74" t="n">
-        <v>357.45</v>
-      </c>
-      <c r="C34" s="62" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="3" t="s">
-        <v>269</v>
-      </c>
-      <c r="B35" s="34" t="n">
-        <f aca="false">B33/B34-1</f>
-        <v>-0.637982981157756</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="30" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="3" t="s">
-        <v>271</v>
-      </c>
-      <c r="B38" s="43" t="n">
-        <f aca="false">K7</f>
-        <v>8935.70507202225</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>272</v>
-      </c>
-      <c r="B39" s="75" t="n">
-        <f aca="false">B25/B38</f>
-        <v>7.09769600861861</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="3" t="s">
-        <v>273</v>
-      </c>
-      <c r="B40" s="76" t="n">
-        <v>10</v>
-      </c>
-      <c r="C40" s="62" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="3" t="s">
-        <v>275</v>
-      </c>
-      <c r="B41" s="43" t="n">
-        <f aca="false">B40*B38</f>
-        <v>89357.0507202225</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="3" t="s">
-        <v>276</v>
-      </c>
-      <c r="B42" s="43" t="n">
-        <f aca="false">B41/(1+B22)^K17</f>
-        <v>31751.3017646748</v>
-      </c>
-    </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="2" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B43" s="38" t="n">
-        <f aca="false">(B24+B42-B29+B30)/B32</f>
-        <v>169.063809657237</v>
+        <f aca="false">$B$41/$B$42</f>
+        <v>121.083756994038</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>278</v>
-      </c>
-      <c r="B44" s="26" t="n">
-        <v>5</v>
+        <v>279</v>
+      </c>
+      <c r="B44" s="75" t="n">
+        <v>357.45</v>
+      </c>
+      <c r="C44" s="62" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
-        <v>279</v>
-      </c>
-      <c r="B45" s="38" t="n">
-        <f aca="false">ROUND(B43/B44,0)*B44</f>
-        <v>170</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="3" t="s">
-        <v>280</v>
-      </c>
-      <c r="B46" s="34" t="n">
-        <f aca="false">B45/B34-1</f>
-        <v>-0.524409008252903</v>
+      <c r="A45" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="B45" s="34" t="n">
+        <f aca="false">$B$43/$B$44-1</f>
+        <v>-0.661256799569064</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="3" t="s">
-        <v>281</v>
-      </c>
-      <c r="B47" s="31" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="C47" s="62" t="s">
+      <c r="A47" s="30" t="s">
         <v>282</v>
       </c>
     </row>
@@ -3094,40 +3162,133 @@
       <c r="A48" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="B48" s="31" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="C48" s="62" t="s">
-        <v>282</v>
+      <c r="B48" s="43" t="n">
+        <f aca="false">K7</f>
+        <v>8935.70507202225</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="2" t="s">
+      <c r="A49" s="3" t="s">
         <v>284</v>
       </c>
-      <c r="B49" s="27" t="str">
-        <f aca="false">IF(B46&gt;B47,"BUY",IF(B46&lt;B48,"SELL","HOLD"))</f>
-        <v>SELL</v>
+      <c r="B49" s="76" t="n">
+        <f aca="false">$B$32/$B$48</f>
+        <v>5.62697940334977</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="B50" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="C50" s="62" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="B51" s="76" t="n">
-        <v>14</v>
-      </c>
-      <c r="C51" s="62" t="s">
-        <v>286</v>
+        <v>287</v>
+      </c>
+      <c r="B51" s="43" t="n">
+        <f aca="false">$B$50*$B$48</f>
+        <v>89357.0507202225</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>287</v>
-      </c>
-      <c r="B52" s="37" t="n">
-        <f aca="false">(B24+B51*B38/(1+B22)^K17-B29+B30)/B32</f>
-        <v>223.724970431371</v>
+        <v>288</v>
+      </c>
+      <c r="B52" s="43" t="n">
+        <f aca="false">$B$51/(1+$B$27)^K22</f>
+        <v>32627.1317364001</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="2" t="s">
+        <v>289</v>
+      </c>
+      <c r="B53" s="38" t="n">
+        <f aca="false">($B$31+$B$52-$B$36+$B$37)*$B$40/$B$42</f>
+        <v>184.336076421551</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>290</v>
+      </c>
+      <c r="B54" s="26" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B55" s="38" t="n">
+        <f aca="false">ROUND($B$53/$B$54,0)*$B$54</f>
+        <v>185</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="3" t="s">
+        <v>292</v>
+      </c>
+      <c r="B56" s="34" t="n">
+        <f aca="false">$B$55/$B$44-1</f>
+        <v>-0.482445097216394</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="3" t="s">
+        <v>293</v>
+      </c>
+      <c r="B57" s="31" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C57" s="62" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="3" t="s">
+        <v>295</v>
+      </c>
+      <c r="B58" s="31" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C58" s="62" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>296</v>
+      </c>
+      <c r="B59" s="27" t="str">
+        <f aca="false">IF($B$56&gt;$B$57,"BUY",IF($B$56&lt;$B$58,"SELL","HOLD"))</f>
+        <v>SELL</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="B61" s="77" t="n">
+        <v>14</v>
+      </c>
+      <c r="C61" s="62" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>299</v>
+      </c>
+      <c r="B62" s="37" t="n">
+        <f aca="false">($B$31+$B$61*$B$48/(1+$B$27)^K22-$B$36+$B$37)*$B$40/$B$42</f>
+        <v>242.192944944847</v>
       </c>
     </row>
   </sheetData>
@@ -3155,17 +3316,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="B4" s="31" t="n">
         <v>0.005</v>
@@ -3173,330 +3334,330 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
-        <v>291</v>
-      </c>
-      <c r="B5" s="76" t="n">
+        <v>303</v>
+      </c>
+      <c r="B5" s="77" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="30" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="27" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="B8" s="65" t="n">
-        <f aca="false">DCF!$B$23+(-2)*$B$4</f>
+        <f aca="false">DCF!$B$28+(-2)*$B$4</f>
         <v>0.03</v>
       </c>
       <c r="C8" s="65" t="n">
-        <f aca="false">DCF!$B$23+(-1)*$B$4</f>
+        <f aca="false">DCF!$B$28+(-1)*$B$4</f>
         <v>0.035</v>
       </c>
       <c r="D8" s="65" t="n">
-        <f aca="false">DCF!$B$23+(0)*$B$4</f>
+        <f aca="false">DCF!$B$28+(0)*$B$4</f>
         <v>0.04</v>
       </c>
       <c r="E8" s="65" t="n">
-        <f aca="false">DCF!$B$23+(1)*$B$4</f>
+        <f aca="false">DCF!$B$28+(1)*$B$4</f>
         <v>0.045</v>
       </c>
       <c r="F8" s="65" t="n">
-        <f aca="false">DCF!$B$23+(2)*$B$4</f>
+        <f aca="false">DCF!$B$28+(2)*$B$4</f>
         <v>0.05</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="66" t="n">
-        <f aca="false">DCF!$B$22+(-2)*$B$4</f>
+        <f aca="false">DCF!$B$27+(-2)*$B$4</f>
         <v>0.1050692</v>
       </c>
       <c r="B9" s="37" t="n">
-        <f aca="false">IF(B$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A9)^DCF!$B$17:$K$17)+DCF!$K$14*(1+B$8)/($A9-B$8)/(1+$A9)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>140.157178523675</v>
+        <f aca="false">IF(B$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A9)^DCF!$B$22:$K$22)+DCF!$K$10*(1+B$8)*(1-B$8/DCF!$B$29)/($A9-B$8)/(1+$A9)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>141.481278112723</v>
       </c>
       <c r="C9" s="37" t="n">
-        <f aca="false">IF(C$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A9)^DCF!$B$17:$K$17)+DCF!$K$14*(1+C$8)/($A9-C$8)/(1+$A9)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>148.16846968373</v>
+        <f aca="false">IF(C$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A9)^DCF!$B$22:$K$22)+DCF!$K$10*(1+C$8)*(1-C$8/DCF!$B$29)/($A9-C$8)/(1+$A9)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>143.132215753428</v>
       </c>
       <c r="D9" s="37" t="n">
-        <f aca="false">IF(D$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A9)^DCF!$B$17:$K$17)+DCF!$K$14*(1+D$8)/($A9-D$8)/(1+$A9)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>157.410956426344</v>
+        <f aca="false">IF(D$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A9)^DCF!$B$22:$K$22)+DCF!$K$10*(1+D$8)*(1-D$8/DCF!$B$29)/($A9-D$8)/(1+$A9)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>144.97554083931</v>
       </c>
       <c r="E9" s="37" t="n">
-        <f aca="false">IF(E$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A9)^DCF!$B$17:$K$17)+DCF!$K$14*(1+E$8)/($A9-E$8)/(1+$A9)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>168.192083061384</v>
+        <f aca="false">IF(E$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A9)^DCF!$B$22:$K$22)+DCF!$K$10*(1+E$8)*(1-E$8/DCF!$B$29)/($A9-E$8)/(1+$A9)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>147.059294823852</v>
       </c>
       <c r="F9" s="37" t="n">
-        <f aca="false">IF(F$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A9)^DCF!$B$17:$K$17)+DCF!$K$14*(1+F$8)/($A9-F$8)/(1+$A9)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>180.930951344212</v>
+        <f aca="false">IF(F$8&gt;=$A9,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A9)^DCF!$B$22:$K$22)+DCF!$K$10*(1+F$8)*(1-F$8/DCF!$B$29)/($A9-F$8)/(1+$A9)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>149.448966827652</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="66" t="n">
-        <f aca="false">DCF!$B$22+(-1)*$B$4</f>
+        <f aca="false">DCF!$B$27+(-1)*$B$4</f>
         <v>0.1100692</v>
       </c>
       <c r="B10" s="37" t="n">
-        <f aca="false">IF(B$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A10)^DCF!$B$17:$K$17)+DCF!$K$14*(1+B$8)/($A10-B$8)/(1+$A10)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>127.922346957083</v>
+        <f aca="false">IF(B$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A10)^DCF!$B$22:$K$22)+DCF!$K$10*(1+B$8)*(1-B$8/DCF!$B$29)/($A10-B$8)/(1+$A10)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>129.905471348028</v>
       </c>
       <c r="C10" s="37" t="n">
-        <f aca="false">IF(C$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A10)^DCF!$B$17:$K$17)+DCF!$K$14*(1+C$8)/($A10-C$8)/(1+$A10)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>134.66916923646</v>
+        <f aca="false">IF(C$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A10)^DCF!$B$22:$K$22)+DCF!$K$10*(1+C$8)*(1-C$8/DCF!$B$29)/($A10-C$8)/(1+$A10)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>130.990241483892</v>
       </c>
       <c r="D10" s="37" t="n">
-        <f aca="false">IF(D$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A10)^DCF!$B$17:$K$17)+DCF!$K$14*(1+D$8)/($A10-D$8)/(1+$A10)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>142.378871394497</v>
+        <f aca="false">IF(D$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A10)^DCF!$B$22:$K$22)+DCF!$K$10*(1+D$8)*(1-D$8/DCF!$B$29)/($A10-D$8)/(1+$A10)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>132.175198939132</v>
       </c>
       <c r="E10" s="37" t="n">
-        <f aca="false">IF(E$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A10)^DCF!$B$17:$K$17)+DCF!$K$14*(1+E$8)/($A10-E$8)/(1+$A10)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>151.273420170908</v>
+        <f aca="false">IF(E$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A10)^DCF!$B$22:$K$22)+DCF!$K$10*(1+E$8)*(1-E$8/DCF!$B$29)/($A10-E$8)/(1+$A10)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>133.483439276481</v>
       </c>
       <c r="F10" s="37" t="n">
-        <f aca="false">IF(F$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A10)^DCF!$B$17:$K$17)+DCF!$K$14*(1+F$8)/($A10-F$8)/(1+$A10)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>161.648685983073</v>
+        <f aca="false">IF(F$8&gt;=$A10,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A10)^DCF!$B$22:$K$22)+DCF!$K$10*(1+F$8)*(1-F$8/DCF!$B$29)/($A10-F$8)/(1+$A10)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>134.945747710853</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="66" t="n">
-        <f aca="false">DCF!$B$22+(0)*$B$4</f>
+        <f aca="false">DCF!$B$27+(0)*$B$4</f>
         <v>0.1150692</v>
       </c>
       <c r="B11" s="37" t="n">
-        <f aca="false">IF(B$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A11)^DCF!$B$17:$K$17)+DCF!$K$14*(1+B$8)/($A11-B$8)/(1+$A11)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>117.178447335938</v>
+        <f aca="false">IF(B$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A11)^DCF!$B$22:$K$22)+DCF!$K$10*(1+B$8)*(1-B$8/DCF!$B$29)/($A11-B$8)/(1+$A11)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>119.717140280606</v>
       </c>
       <c r="C11" s="37" t="n">
-        <f aca="false">IF(C$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A11)^DCF!$B$17:$K$17)+DCF!$K$14*(1+C$8)/($A11-C$8)/(1+$A11)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>122.909028767913</v>
+        <f aca="false">IF(C$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A11)^DCF!$B$22:$K$22)+DCF!$K$10*(1+C$8)*(1-C$8/DCF!$B$29)/($A11-C$8)/(1+$A11)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>120.380707675442</v>
       </c>
       <c r="D11" s="38" t="n">
-        <f aca="false">IF(D$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A11)^DCF!$B$17:$K$17)+DCF!$K$14*(1+D$8)/($A11-D$8)/(1+$A11)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>129.40298338516</v>
+        <f aca="false">IF(D$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A11)^DCF!$B$22:$K$22)+DCF!$K$10*(1+D$8)*(1-D$8/DCF!$B$29)/($A11-D$8)/(1+$A11)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>121.083756994038</v>
       </c>
       <c r="E11" s="37" t="n">
-        <f aca="false">IF(E$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A11)^DCF!$B$17:$K$17)+DCF!$K$14*(1+E$8)/($A11-E$8)/(1+$A11)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>136.823729605172</v>
+        <f aca="false">IF(E$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A11)^DCF!$B$22:$K$22)+DCF!$K$10*(1+E$8)*(1-E$8/DCF!$B$29)/($A11-E$8)/(1+$A11)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>121.834740293165</v>
       </c>
       <c r="F11" s="37" t="n">
-        <f aca="false">IF(F$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A11)^DCF!$B$17:$K$17)+DCF!$K$14*(1+F$8)/($A11-F$8)/(1+$A11)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>145.384914960753</v>
+        <f aca="false">IF(F$8&gt;=$A11,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A11)^DCF!$B$22:$K$22)+DCF!$K$10*(1+F$8)*(1-F$8/DCF!$B$29)/($A11-F$8)/(1+$A11)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>122.644707496719</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="66" t="n">
-        <f aca="false">DCF!$B$22+(1)*$B$4</f>
+        <f aca="false">DCF!$B$27+(1)*$B$4</f>
         <v>0.1200692</v>
       </c>
       <c r="B12" s="37" t="n">
-        <f aca="false">IF(B$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A12)^DCF!$B$17:$K$17)+DCF!$K$14*(1+B$8)/($A12-B$8)/(1+$A12)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>107.676080894372</v>
+        <f aca="false">IF(B$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A12)^DCF!$B$22:$K$22)+DCF!$K$10*(1+B$8)*(1-B$8/DCF!$B$29)/($A12-B$8)/(1+$A12)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>110.685176331286</v>
       </c>
       <c r="C12" s="37" t="n">
-        <f aca="false">IF(C$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A12)^DCF!$B$17:$K$17)+DCF!$K$14*(1+C$8)/($A12-C$8)/(1+$A12)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>112.580324958075</v>
+        <f aca="false">IF(C$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A12)^DCF!$B$22:$K$22)+DCF!$K$10*(1+C$8)*(1-C$8/DCF!$B$29)/($A12-C$8)/(1+$A12)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>111.033906635952</v>
       </c>
       <c r="D12" s="37" t="n">
-        <f aca="false">IF(D$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A12)^DCF!$B$17:$K$17)+DCF!$K$14*(1+D$8)/($A12-D$8)/(1+$A12)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>118.097069716641</v>
+        <f aca="false">IF(D$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A12)^DCF!$B$22:$K$22)+DCF!$K$10*(1+D$8)*(1-D$8/DCF!$B$29)/($A12-D$8)/(1+$A12)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>111.382191856473</v>
       </c>
       <c r="E12" s="37" t="n">
-        <f aca="false">IF(E$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A12)^DCF!$B$17:$K$17)+DCF!$K$14*(1+E$8)/($A12-E$8)/(1+$A12)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>124.348702386435</v>
+        <f aca="false">IF(E$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A12)^DCF!$B$22:$K$22)+DCF!$K$10*(1+E$8)*(1-E$8/DCF!$B$29)/($A12-E$8)/(1+$A12)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>111.729943058076</v>
       </c>
       <c r="F12" s="37" t="n">
-        <f aca="false">IF(F$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A12)^DCF!$B$17:$K$17)+DCF!$K$14*(1+F$8)/($A12-F$8)/(1+$A12)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>131.492543425927</v>
+        <f aca="false">IF(F$8&gt;=$A12,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A12)^DCF!$B$22:$K$22)+DCF!$K$10*(1+F$8)*(1-F$8/DCF!$B$29)/($A12-F$8)/(1+$A12)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>112.077045921151</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="66" t="n">
-        <f aca="false">DCF!$B$22+(2)*$B$4</f>
+        <f aca="false">DCF!$B$27+(2)*$B$4</f>
         <v>0.1250692</v>
       </c>
       <c r="B13" s="37" t="n">
-        <f aca="false">IF(B$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A13)^DCF!$B$17:$K$17)+DCF!$K$14*(1+B$8)/($A13-B$8)/(1+$A13)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>99.2183472517214</v>
+        <f aca="false">IF(B$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A13)^DCF!$B$22:$K$22)+DCF!$K$10*(1+B$8)*(1-B$8/DCF!$B$29)/($A13-B$8)/(1+$A13)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>102.627071137506</v>
       </c>
       <c r="C13" s="37" t="n">
-        <f aca="false">IF(C$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A13)^DCF!$B$17:$K$17)+DCF!$K$14*(1+C$8)/($A13-C$8)/(1+$A13)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>103.443693953947</v>
+        <f aca="false">IF(C$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A13)^DCF!$B$22:$K$22)+DCF!$K$10*(1+C$8)*(1-C$8/DCF!$B$29)/($A13-C$8)/(1+$A13)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>102.739973238036</v>
       </c>
       <c r="D13" s="37" t="n">
-        <f aca="false">IF(D$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A13)^DCF!$B$17:$K$17)+DCF!$K$14*(1+D$8)/($A13-D$8)/(1+$A13)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>108.165735899836</v>
+        <f aca="false">IF(D$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A13)^DCF!$B$22:$K$22)+DCF!$K$10*(1+D$8)*(1-D$8/DCF!$B$29)/($A13-D$8)/(1+$A13)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>102.826406058116</v>
       </c>
       <c r="E13" s="37" t="n">
-        <f aca="false">IF(E$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A13)^DCF!$B$17:$K$17)+DCF!$K$14*(1+E$8)/($A13-E$8)/(1+$A13)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>113.477522959438</v>
+        <f aca="false">IF(E$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A13)^DCF!$B$22:$K$22)+DCF!$K$10*(1+E$8)*(1-E$8/DCF!$B$29)/($A13-E$8)/(1+$A13)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>102.881410896938</v>
       </c>
       <c r="F13" s="37" t="n">
-        <f aca="false">IF(F$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A13)^DCF!$B$17:$K$17)+DCF!$K$14*(1+F$8)/($A13-F$8)/(1+$A13)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32)</f>
-        <v>119.496895428183</v>
+        <f aca="false">IF(F$8&gt;=$A13,NA(),(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A13)^DCF!$B$22:$K$22)+DCF!$K$10*(1+F$8)*(1-F$8/DCF!$B$29)/($A13-F$8)/(1+$A13)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42)</f>
+        <v>102.898707952413</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="30" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="27" t="s">
-        <v>295</v>
-      </c>
-      <c r="B16" s="77" t="n">
-        <f aca="false">DCF!$B$40+(-2)*$B$5</f>
+        <v>307</v>
+      </c>
+      <c r="B16" s="78" t="n">
+        <f aca="false">DCF!$B$50+(-2)*$B$5</f>
         <v>6</v>
       </c>
-      <c r="C16" s="77" t="n">
-        <f aca="false">DCF!$B$40+(-1)*$B$5</f>
+      <c r="C16" s="78" t="n">
+        <f aca="false">DCF!$B$50+(-1)*$B$5</f>
         <v>8</v>
       </c>
-      <c r="D16" s="77" t="n">
-        <f aca="false">DCF!$B$40+(0)*$B$5</f>
+      <c r="D16" s="78" t="n">
+        <f aca="false">DCF!$B$50+(0)*$B$5</f>
         <v>10</v>
       </c>
-      <c r="E16" s="77" t="n">
-        <f aca="false">DCF!$B$40+(1)*$B$5</f>
+      <c r="E16" s="78" t="n">
+        <f aca="false">DCF!$B$50+(1)*$B$5</f>
         <v>12</v>
       </c>
-      <c r="F16" s="77" t="n">
-        <f aca="false">DCF!$B$40+(2)*$B$5</f>
+      <c r="F16" s="78" t="n">
+        <f aca="false">DCF!$B$50+(2)*$B$5</f>
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="66" t="n">
-        <f aca="false">DCF!$B$22+(-2)*$B$4</f>
+        <f aca="false">DCF!$B$27+(-2)*$B$4</f>
         <v>0.1050692</v>
       </c>
       <c r="B17" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A17)^DCF!$B$17:$K$17)+B$16*DCF!$B$38/(1+$A17)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>124.832514997476</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A17)^DCF!$B$22:$K$22)+B$16*DCF!$B$48/(1+$A17)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>137.244689743407</v>
       </c>
       <c r="C17" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A17)^DCF!$B$17:$K$17)+C$16*DCF!$B$38/(1+$A17)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>154.605072053205</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A17)^DCF!$B$22:$K$22)+C$16*DCF!$B$48/(1+$A17)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>168.68702493657</v>
       </c>
       <c r="D17" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A17)^DCF!$B$17:$K$17)+D$16*DCF!$B$38/(1+$A17)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>184.377629108933</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A17)^DCF!$B$22:$K$22)+D$16*DCF!$B$48/(1+$A17)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>200.129360129733</v>
       </c>
       <c r="E17" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A17)^DCF!$B$17:$K$17)+E$16*DCF!$B$38/(1+$A17)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>214.150186164662</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A17)^DCF!$B$22:$K$22)+E$16*DCF!$B$48/(1+$A17)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>231.571695322896</v>
       </c>
       <c r="F17" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A17)^DCF!$B$17:$K$17)+F$16*DCF!$B$38/(1+$A17)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>243.92274322039</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A17)^DCF!$B$22:$K$22)+F$16*DCF!$B$48/(1+$A17)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>263.014030516059</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="66" t="n">
-        <f aca="false">DCF!$B$22+(-1)*$B$4</f>
+        <f aca="false">DCF!$B$27+(-1)*$B$4</f>
         <v>0.1100692</v>
       </c>
       <c r="B18" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A18)^DCF!$B$17:$K$17)+B$16*DCF!$B$38/(1+$A18)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>119.501189687698</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A18)^DCF!$B$22:$K$22)+B$16*DCF!$B$48/(1+$A18)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>131.745326438666</v>
       </c>
       <c r="C18" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A18)^DCF!$B$17:$K$17)+C$16*DCF!$B$38/(1+$A18)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>148.023890255743</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A18)^DCF!$B$22:$K$22)+C$16*DCF!$B$48/(1+$A18)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>161.901699605484</v>
       </c>
       <c r="D18" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A18)^DCF!$B$17:$K$17)+D$16*DCF!$B$38/(1+$A18)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>176.546590823789</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A18)^DCF!$B$22:$K$22)+D$16*DCF!$B$48/(1+$A18)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>192.058072772303</v>
       </c>
       <c r="E18" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A18)^DCF!$B$17:$K$17)+E$16*DCF!$B$38/(1+$A18)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>205.069291391834</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A18)^DCF!$B$22:$K$22)+E$16*DCF!$B$48/(1+$A18)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>222.214445939122</v>
       </c>
       <c r="F18" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A18)^DCF!$B$17:$K$17)+F$16*DCF!$B$38/(1+$A18)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>233.591991959879</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A18)^DCF!$B$22:$K$22)+F$16*DCF!$B$48/(1+$A18)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>252.370819105941</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="66" t="n">
-        <f aca="false">DCF!$B$22+(0)*$B$4</f>
+        <f aca="false">DCF!$B$27+(0)*$B$4</f>
         <v>0.1150692</v>
       </c>
       <c r="B19" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A19)^DCF!$B$17:$K$17)+B$16*DCF!$B$38/(1+$A19)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>114.402648883104</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A19)^DCF!$B$22:$K$22)+B$16*DCF!$B$48/(1+$A19)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>126.479207898256</v>
       </c>
       <c r="C19" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A19)^DCF!$B$17:$K$17)+C$16*DCF!$B$38/(1+$A19)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>141.73322927017</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A19)^DCF!$B$22:$K$22)+C$16*DCF!$B$48/(1+$A19)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>155.407642159904</v>
       </c>
       <c r="D19" s="38" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A19)^DCF!$B$17:$K$17)+D$16*DCF!$B$38/(1+$A19)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>169.063809657237</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A19)^DCF!$B$22:$K$22)+D$16*DCF!$B$48/(1+$A19)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>184.336076421551</v>
       </c>
       <c r="E19" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A19)^DCF!$B$17:$K$17)+E$16*DCF!$B$38/(1+$A19)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>196.394390044304</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A19)^DCF!$B$22:$K$22)+E$16*DCF!$B$48/(1+$A19)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>213.264510683199</v>
       </c>
       <c r="F19" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A19)^DCF!$B$17:$K$17)+F$16*DCF!$B$38/(1+$A19)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>223.724970431371</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A19)^DCF!$B$22:$K$22)+F$16*DCF!$B$48/(1+$A19)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>242.192944944847</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="66" t="n">
-        <f aca="false">DCF!$B$22+(1)*$B$4</f>
+        <f aca="false">DCF!$B$27+(1)*$B$4</f>
         <v>0.1200692</v>
       </c>
       <c r="B20" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A20)^DCF!$B$17:$K$17)+B$16*DCF!$B$38/(1+$A20)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>109.525664565478</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A20)^DCF!$B$22:$K$22)+B$16*DCF!$B$48/(1+$A20)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>121.435330806186</v>
       </c>
       <c r="C20" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A20)^DCF!$B$17:$K$17)+C$16*DCF!$B$38/(1+$A20)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>135.718952812982</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A20)^DCF!$B$22:$K$22)+C$16*DCF!$B$48/(1+$A20)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>149.190988475413</v>
       </c>
       <c r="D20" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A20)^DCF!$B$17:$K$17)+D$16*DCF!$B$38/(1+$A20)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>161.912241060486</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A20)^DCF!$B$22:$K$22)+D$16*DCF!$B$48/(1+$A20)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>176.94664614464</v>
       </c>
       <c r="E20" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A20)^DCF!$B$17:$K$17)+E$16*DCF!$B$38/(1+$A20)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>188.10552930799</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A20)^DCF!$B$22:$K$22)+E$16*DCF!$B$48/(1+$A20)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>204.702303813867</v>
       </c>
       <c r="F20" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A20)^DCF!$B$17:$K$17)+F$16*DCF!$B$38/(1+$A20)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>214.298817555494</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A20)^DCF!$B$22:$K$22)+F$16*DCF!$B$48/(1+$A20)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>232.457961483094</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="66" t="n">
-        <f aca="false">DCF!$B$22+(2)*$B$4</f>
+        <f aca="false">DCF!$B$27+(2)*$B$4</f>
         <v>0.1250692</v>
       </c>
       <c r="B21" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A21)^DCF!$B$17:$K$17)+B$16*DCF!$B$38/(1+$A21)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>104.859602546607</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A21)^DCF!$B$22:$K$22)+B$16*DCF!$B$48/(1+$A21)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>116.603262569662</v>
       </c>
       <c r="C21" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A21)^DCF!$B$17:$K$17)+C$16*DCF!$B$38/(1+$A21)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>129.967676966441</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A21)^DCF!$B$22:$K$22)+C$16*DCF!$B$48/(1+$A21)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>143.238598067401</v>
       </c>
       <c r="D21" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A21)^DCF!$B$17:$K$17)+D$16*DCF!$B$38/(1+$A21)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>155.075751386274</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A21)^DCF!$B$22:$K$22)+D$16*DCF!$B$48/(1+$A21)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>169.87393356514</v>
       </c>
       <c r="E21" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A21)^DCF!$B$17:$K$17)+E$16*DCF!$B$38/(1+$A21)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>180.183825806107</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A21)^DCF!$B$22:$K$22)+E$16*DCF!$B$48/(1+$A21)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>196.509269062879</v>
       </c>
       <c r="F21" s="37" t="n">
-        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,1/(1+$A21)^DCF!$B$17:$K$17)+F$16*DCF!$B$38/(1+$A21)^DCF!$K$17-DCF!$B$29+DCF!$B$30)/DCF!$B$32</f>
-        <v>205.291900225941</v>
+        <f aca="false">(SUMPRODUCT(DCF!$B$14:$K$14,DCF!$B$21:$K$21,1/(1+$A21)^DCF!$B$22:$K$22)+F$16*DCF!$B$48/(1+$A21)^DCF!$K$22-DCF!$B$36+DCF!$B$37)*DCF!$B$40/DCF!$B$42</f>
+        <v>223.144604560618</v>
       </c>
     </row>
   </sheetData>
@@ -3524,7 +3685,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3599,7 +3760,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="B5" s="14"/>
       <c r="C5" s="14"/>
@@ -3624,347 +3785,347 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>298</v>
-      </c>
-      <c r="B6" s="78" t="n">
+        <v>310</v>
+      </c>
+      <c r="B6" s="79" t="n">
         <f aca="false">('Balance Sheet'!B13-'Balance Sheet'!B22)</f>
         <v>0</v>
       </c>
-      <c r="C6" s="78" t="n">
+      <c r="C6" s="79" t="n">
         <f aca="false">('Balance Sheet'!C13-'Balance Sheet'!C22)</f>
         <v>0</v>
       </c>
-      <c r="D6" s="78" t="n">
+      <c r="D6" s="79" t="n">
         <f aca="false">('Balance Sheet'!D13-'Balance Sheet'!D22)</f>
         <v>0</v>
       </c>
-      <c r="E6" s="78" t="n">
+      <c r="E6" s="79" t="n">
         <f aca="false">('Balance Sheet'!E13-'Balance Sheet'!E22)</f>
         <v>0</v>
       </c>
-      <c r="F6" s="78" t="n">
+      <c r="F6" s="79" t="n">
         <f aca="false">('Balance Sheet'!F13-'Balance Sheet'!F22)</f>
         <v>0</v>
       </c>
-      <c r="G6" s="78" t="n">
+      <c r="G6" s="79" t="n">
         <f aca="false">('Balance Sheet'!G13-'Balance Sheet'!G22)</f>
         <v>0</v>
       </c>
-      <c r="H6" s="78" t="n">
+      <c r="H6" s="79" t="n">
         <f aca="false">('Balance Sheet'!H13-'Balance Sheet'!H22)</f>
         <v>0</v>
       </c>
-      <c r="I6" s="78" t="n">
+      <c r="I6" s="79" t="n">
         <f aca="false">('Balance Sheet'!I13-'Balance Sheet'!I22)</f>
         <v>0</v>
       </c>
-      <c r="J6" s="78" t="n">
+      <c r="J6" s="79" t="n">
         <f aca="false">('Balance Sheet'!J13-'Balance Sheet'!J22)</f>
         <v>0</v>
       </c>
-      <c r="K6" s="78" t="n">
+      <c r="K6" s="79" t="n">
         <f aca="false">('Balance Sheet'!K13-'Balance Sheet'!K22)</f>
         <v>0</v>
       </c>
-      <c r="L6" s="78" t="n">
+      <c r="L6" s="79" t="n">
         <f aca="false">('Balance Sheet'!L13-'Balance Sheet'!L22)</f>
         <v>0</v>
       </c>
-      <c r="M6" s="78" t="n">
+      <c r="M6" s="79" t="n">
         <f aca="false">('Balance Sheet'!M13-'Balance Sheet'!M22)</f>
         <v>0</v>
       </c>
-      <c r="N6" s="78" t="n">
+      <c r="N6" s="79" t="n">
         <f aca="false">('Balance Sheet'!N13-'Balance Sheet'!N22)</f>
         <v>0</v>
       </c>
-      <c r="O6" s="78" t="n">
+      <c r="O6" s="79" t="n">
         <f aca="false">('Balance Sheet'!O13-'Balance Sheet'!O22)</f>
         <v>0</v>
       </c>
-      <c r="P6" s="78" t="n">
+      <c r="P6" s="79" t="n">
         <f aca="false">('Balance Sheet'!P13-'Balance Sheet'!P22)</f>
         <v>0</v>
       </c>
-      <c r="Q6" s="78" t="n">
+      <c r="Q6" s="79" t="n">
         <f aca="false">('Balance Sheet'!Q13-'Balance Sheet'!Q22)</f>
         <v>0</v>
       </c>
-      <c r="R6" s="78" t="n">
+      <c r="R6" s="79" t="n">
         <f aca="false">('Balance Sheet'!R13-'Balance Sheet'!R22)</f>
         <v>0</v>
       </c>
-      <c r="S6" s="78" t="n">
+      <c r="S6" s="79" t="n">
         <f aca="false">('Balance Sheet'!S13-'Balance Sheet'!S22)</f>
         <v>0</v>
       </c>
-      <c r="T6" s="78" t="n">
+      <c r="T6" s="79" t="n">
         <f aca="false">('Balance Sheet'!T13-'Balance Sheet'!T22)</f>
         <v>0</v>
       </c>
-      <c r="U6" s="78" t="n">
+      <c r="U6" s="79" t="n">
         <f aca="false">('Balance Sheet'!U13-'Balance Sheet'!U22)</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>299</v>
-      </c>
-      <c r="B7" s="78" t="n">
+        <v>311</v>
+      </c>
+      <c r="B7" s="79" t="n">
         <f aca="false">('Balance Sheet'!B6-'Cash Flow'!B23)</f>
         <v>-1268.7</v>
       </c>
-      <c r="C7" s="78" t="n">
+      <c r="C7" s="79" t="n">
         <f aca="false">('Balance Sheet'!C6-'Cash Flow'!C23)</f>
         <v>491.16</v>
       </c>
-      <c r="D7" s="78" t="n">
+      <c r="D7" s="79" t="n">
         <f aca="false">('Balance Sheet'!D6-'Cash Flow'!D23)</f>
         <v>7.87999999999984</v>
       </c>
-      <c r="E7" s="78" t="n">
+      <c r="E7" s="79" t="n">
         <f aca="false">('Balance Sheet'!E6-'Cash Flow'!E23)</f>
         <v>-529.87</v>
       </c>
-      <c r="F7" s="78" t="n">
+      <c r="F7" s="79" t="n">
         <f aca="false">('Balance Sheet'!F6-'Cash Flow'!F23)</f>
         <v>51.5699999999998</v>
       </c>
-      <c r="G7" s="78" t="n">
+      <c r="G7" s="79" t="n">
         <f aca="false">('Balance Sheet'!G6-'Cash Flow'!G23)</f>
         <v>53</v>
       </c>
-      <c r="H7" s="78" t="n">
+      <c r="H7" s="79" t="n">
         <f aca="false">('Balance Sheet'!H6-'Cash Flow'!H23)</f>
         <v>-17.3399999999992</v>
       </c>
-      <c r="I7" s="78" t="n">
+      <c r="I7" s="79" t="n">
         <f aca="false">('Balance Sheet'!I6-'Cash Flow'!I23)</f>
         <v>2988.66</v>
       </c>
-      <c r="J7" s="78" t="n">
+      <c r="J7" s="79" t="n">
         <f aca="false">('Balance Sheet'!J6-'Cash Flow'!J23)</f>
         <v>333.339999999999</v>
       </c>
-      <c r="K7" s="78" t="n">
+      <c r="K7" s="79" t="n">
         <f aca="false">('Balance Sheet'!K6-'Cash Flow'!K23)</f>
         <v>-155.04</v>
       </c>
-      <c r="L7" s="78" t="n">
+      <c r="L7" s="79" t="n">
         <f aca="false">('Balance Sheet'!L6-'Cash Flow'!L23)</f>
         <v>0</v>
       </c>
-      <c r="M7" s="78" t="n">
+      <c r="M7" s="79" t="n">
         <f aca="false">('Balance Sheet'!M6-'Cash Flow'!M23)</f>
         <v>0</v>
       </c>
-      <c r="N7" s="78" t="n">
+      <c r="N7" s="79" t="n">
         <f aca="false">('Balance Sheet'!N6-'Cash Flow'!N23)</f>
         <v>0</v>
       </c>
-      <c r="O7" s="78" t="n">
+      <c r="O7" s="79" t="n">
         <f aca="false">('Balance Sheet'!O6-'Cash Flow'!O23)</f>
         <v>0</v>
       </c>
-      <c r="P7" s="78" t="n">
+      <c r="P7" s="79" t="n">
         <f aca="false">('Balance Sheet'!P6-'Cash Flow'!P23)</f>
         <v>0</v>
       </c>
-      <c r="Q7" s="78" t="n">
+      <c r="Q7" s="79" t="n">
         <f aca="false">('Balance Sheet'!Q6-'Cash Flow'!Q23)</f>
         <v>0</v>
       </c>
-      <c r="R7" s="78" t="n">
+      <c r="R7" s="79" t="n">
         <f aca="false">('Balance Sheet'!R6-'Cash Flow'!R23)</f>
         <v>0</v>
       </c>
-      <c r="S7" s="78" t="n">
+      <c r="S7" s="79" t="n">
         <f aca="false">('Balance Sheet'!S6-'Cash Flow'!S23)</f>
         <v>0</v>
       </c>
-      <c r="T7" s="78" t="n">
+      <c r="T7" s="79" t="n">
         <f aca="false">('Balance Sheet'!T6-'Cash Flow'!T23)</f>
         <v>0</v>
       </c>
-      <c r="U7" s="78" t="n">
+      <c r="U7" s="79" t="n">
         <f aca="false">('Balance Sheet'!U6-'Cash Flow'!U23)</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>300</v>
-      </c>
-      <c r="B8" s="78" t="n">
+        <v>312</v>
+      </c>
+      <c r="B8" s="79" t="n">
         <f aca="false">('Balance Sheet'!B16-(((0+'Income Statement'!B18)-Schedules!B22)+Drivers!B27))</f>
         <v>1487.52</v>
       </c>
-      <c r="C8" s="78" t="n">
+      <c r="C8" s="79" t="n">
         <f aca="false">('Balance Sheet'!C16-((('Balance Sheet'!B16+'Income Statement'!C18)-Schedules!C22)+Drivers!C27))</f>
         <v>487.3</v>
       </c>
-      <c r="D8" s="78" t="n">
+      <c r="D8" s="79" t="n">
         <f aca="false">('Balance Sheet'!D16-((('Balance Sheet'!C16+'Income Statement'!D18)-Schedules!D22)+Drivers!D27))</f>
         <v>7.88000000000011</v>
       </c>
-      <c r="E8" s="78" t="n">
+      <c r="E8" s="79" t="n">
         <f aca="false">('Balance Sheet'!E16-((('Balance Sheet'!D16+'Income Statement'!E18)-Schedules!E22)+Drivers!E27))</f>
         <v>-529.62</v>
       </c>
-      <c r="F8" s="78" t="n">
+      <c r="F8" s="79" t="n">
         <f aca="false">('Balance Sheet'!F16-((('Balance Sheet'!E16+'Income Statement'!F18)-Schedules!F22)+Drivers!F27))</f>
         <v>51.5699999999997</v>
       </c>
-      <c r="G8" s="78" t="n">
+      <c r="G8" s="79" t="n">
         <f aca="false">('Balance Sheet'!G16-((('Balance Sheet'!F16+'Income Statement'!G18)-Schedules!G22)+Drivers!G27))</f>
         <v>53.0000000000005</v>
       </c>
-      <c r="H8" s="78" t="n">
+      <c r="H8" s="79" t="n">
         <f aca="false">('Balance Sheet'!H16-((('Balance Sheet'!G16+'Income Statement'!H18)-Schedules!H22)+Drivers!H27))</f>
         <v>-316.98</v>
       </c>
-      <c r="I8" s="78" t="n">
+      <c r="I8" s="79" t="n">
         <f aca="false">('Balance Sheet'!I16-((('Balance Sheet'!H16+'Income Statement'!I18)-Schedules!I22)+Drivers!I27))</f>
         <v>2937.93</v>
       </c>
-      <c r="J8" s="78" t="n">
+      <c r="J8" s="79" t="n">
         <f aca="false">('Balance Sheet'!J16-((('Balance Sheet'!I16+'Income Statement'!J18)-Schedules!J22)+Drivers!J27))</f>
         <v>328.940000000001</v>
       </c>
-      <c r="K8" s="78" t="n">
+      <c r="K8" s="79" t="n">
         <f aca="false">('Balance Sheet'!K16-((('Balance Sheet'!J16+'Income Statement'!K18)-Schedules!K22)+Drivers!K27))</f>
         <v>-157.380000000001</v>
       </c>
-      <c r="L8" s="78" t="n">
+      <c r="L8" s="79" t="n">
         <f aca="false">('Balance Sheet'!L16-((('Balance Sheet'!K16+'Income Statement'!L18)-Schedules!L22)+Drivers!L27))</f>
         <v>0</v>
       </c>
-      <c r="M8" s="78" t="n">
+      <c r="M8" s="79" t="n">
         <f aca="false">('Balance Sheet'!M16-((('Balance Sheet'!L16+'Income Statement'!M18)-Schedules!M22)+Drivers!M27))</f>
         <v>0</v>
       </c>
-      <c r="N8" s="78" t="n">
+      <c r="N8" s="79" t="n">
         <f aca="false">('Balance Sheet'!N16-((('Balance Sheet'!M16+'Income Statement'!N18)-Schedules!N22)+Drivers!N27))</f>
         <v>0</v>
       </c>
-      <c r="O8" s="78" t="n">
+      <c r="O8" s="79" t="n">
         <f aca="false">('Balance Sheet'!O16-((('Balance Sheet'!N16+'Income Statement'!O18)-Schedules!O22)+Drivers!O27))</f>
         <v>0</v>
       </c>
-      <c r="P8" s="78" t="n">
+      <c r="P8" s="79" t="n">
         <f aca="false">('Balance Sheet'!P16-((('Balance Sheet'!O16+'Income Statement'!P18)-Schedules!P22)+Drivers!P27))</f>
         <v>0</v>
       </c>
-      <c r="Q8" s="78" t="n">
+      <c r="Q8" s="79" t="n">
         <f aca="false">('Balance Sheet'!Q16-((('Balance Sheet'!P16+'Income Statement'!Q18)-Schedules!Q22)+Drivers!Q27))</f>
         <v>0</v>
       </c>
-      <c r="R8" s="78" t="n">
+      <c r="R8" s="79" t="n">
         <f aca="false">('Balance Sheet'!R16-((('Balance Sheet'!Q16+'Income Statement'!R18)-Schedules!R22)+Drivers!R27))</f>
         <v>0</v>
       </c>
-      <c r="S8" s="78" t="n">
+      <c r="S8" s="79" t="n">
         <f aca="false">('Balance Sheet'!S16-((('Balance Sheet'!R16+'Income Statement'!S18)-Schedules!S22)+Drivers!S27))</f>
         <v>0</v>
       </c>
-      <c r="T8" s="78" t="n">
+      <c r="T8" s="79" t="n">
         <f aca="false">('Balance Sheet'!T16-((('Balance Sheet'!S16+'Income Statement'!T18)-Schedules!T22)+Drivers!T27))</f>
         <v>0</v>
       </c>
-      <c r="U8" s="78" t="n">
+      <c r="U8" s="79" t="n">
         <f aca="false">('Balance Sheet'!U16-((('Balance Sheet'!T16+'Income Statement'!U18)-Schedules!U22)+Drivers!U27))</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>301</v>
-      </c>
-      <c r="B9" s="78" t="n">
+        <v>313</v>
+      </c>
+      <c r="B9" s="79" t="n">
         <f aca="false">('Balance Sheet'!B10-Schedules!B9)</f>
         <v>2812.54</v>
       </c>
-      <c r="C9" s="78" t="n">
+      <c r="C9" s="79" t="n">
         <f aca="false">('Balance Sheet'!C10-Schedules!C9)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="78" t="n">
+      <c r="D9" s="79" t="n">
         <f aca="false">('Balance Sheet'!D10-Schedules!D9)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="78" t="n">
+      <c r="E9" s="79" t="n">
         <f aca="false">('Balance Sheet'!E10-Schedules!E9)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="78" t="n">
+      <c r="F9" s="79" t="n">
         <f aca="false">('Balance Sheet'!F10-Schedules!F9)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="78" t="n">
+      <c r="G9" s="79" t="n">
         <f aca="false">('Balance Sheet'!G10-Schedules!G9)</f>
         <v>0</v>
       </c>
-      <c r="H9" s="78" t="n">
+      <c r="H9" s="79" t="n">
         <f aca="false">('Balance Sheet'!H10-Schedules!H9)</f>
         <v>0</v>
       </c>
-      <c r="I9" s="78" t="n">
+      <c r="I9" s="79" t="n">
         <f aca="false">('Balance Sheet'!I10-Schedules!I9)</f>
         <v>0</v>
       </c>
-      <c r="J9" s="78" t="n">
+      <c r="J9" s="79" t="n">
         <f aca="false">('Balance Sheet'!J10-Schedules!J9)</f>
         <v>0</v>
       </c>
-      <c r="K9" s="78" t="n">
+      <c r="K9" s="79" t="n">
         <f aca="false">('Balance Sheet'!K10-Schedules!K9)</f>
         <v>0</v>
       </c>
-      <c r="L9" s="78" t="n">
+      <c r="L9" s="79" t="n">
         <f aca="false">('Balance Sheet'!L10-Schedules!L9)</f>
         <v>0</v>
       </c>
-      <c r="M9" s="78" t="n">
+      <c r="M9" s="79" t="n">
         <f aca="false">('Balance Sheet'!M10-Schedules!M9)</f>
         <v>0</v>
       </c>
-      <c r="N9" s="78" t="n">
+      <c r="N9" s="79" t="n">
         <f aca="false">('Balance Sheet'!N10-Schedules!N9)</f>
         <v>0</v>
       </c>
-      <c r="O9" s="78" t="n">
+      <c r="O9" s="79" t="n">
         <f aca="false">('Balance Sheet'!O10-Schedules!O9)</f>
         <v>0</v>
       </c>
-      <c r="P9" s="78" t="n">
+      <c r="P9" s="79" t="n">
         <f aca="false">('Balance Sheet'!P10-Schedules!P9)</f>
         <v>0</v>
       </c>
-      <c r="Q9" s="78" t="n">
+      <c r="Q9" s="79" t="n">
         <f aca="false">('Balance Sheet'!Q10-Schedules!Q9)</f>
         <v>0</v>
       </c>
-      <c r="R9" s="78" t="n">
+      <c r="R9" s="79" t="n">
         <f aca="false">('Balance Sheet'!R10-Schedules!R9)</f>
         <v>0</v>
       </c>
-      <c r="S9" s="78" t="n">
+      <c r="S9" s="79" t="n">
         <f aca="false">('Balance Sheet'!S10-Schedules!S9)</f>
         <v>0</v>
       </c>
-      <c r="T9" s="78" t="n">
+      <c r="T9" s="79" t="n">
         <f aca="false">('Balance Sheet'!T10-Schedules!T9)</f>
         <v>0</v>
       </c>
-      <c r="U9" s="78" t="n">
+      <c r="U9" s="79" t="n">
         <f aca="false">('Balance Sheet'!U10-Schedules!U9)</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="B10" s="14"/>
       <c r="C10" s="14"/>
@@ -3989,255 +4150,255 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>303</v>
-      </c>
-      <c r="B11" s="78" t="n">
+        <v>315</v>
+      </c>
+      <c r="B11" s="79" t="n">
         <f aca="false">('Balance Sheet'!B6-Drivers!B29)</f>
         <v>44.88</v>
       </c>
-      <c r="C11" s="78" t="n">
+      <c r="C11" s="79" t="n">
         <f aca="false">('Balance Sheet'!C6-Drivers!C29)</f>
         <v>328.45</v>
       </c>
-      <c r="D11" s="78" t="n">
+      <c r="D11" s="79" t="n">
         <f aca="false">('Balance Sheet'!D6-Drivers!D29)</f>
         <v>101.76</v>
       </c>
-      <c r="E11" s="78" t="n">
+      <c r="E11" s="79" t="n">
         <f aca="false">('Balance Sheet'!E6-Drivers!E29)</f>
         <v>162.61</v>
       </c>
-      <c r="F11" s="78" t="n">
+      <c r="F11" s="79" t="n">
         <f aca="false">('Balance Sheet'!F6-Drivers!F29)</f>
         <v>314.48</v>
       </c>
-      <c r="G11" s="78" t="n">
+      <c r="G11" s="79" t="n">
         <f aca="false">('Balance Sheet'!G6-Drivers!G29)</f>
         <v>1038.24</v>
       </c>
-      <c r="H11" s="78" t="n">
+      <c r="H11" s="79" t="n">
         <f aca="false">('Balance Sheet'!H6-Drivers!H29)</f>
         <v>1631.64</v>
       </c>
-      <c r="I11" s="78" t="n">
+      <c r="I11" s="79" t="n">
         <f aca="false">('Balance Sheet'!I6-Drivers!I29)</f>
         <v>4090.22</v>
       </c>
-      <c r="J11" s="78" t="n">
+      <c r="J11" s="79" t="n">
         <f aca="false">('Balance Sheet'!J6-Drivers!J29)</f>
         <v>2482.07</v>
       </c>
-      <c r="K11" s="78" t="n">
+      <c r="K11" s="79" t="n">
         <f aca="false">('Balance Sheet'!K6-Drivers!K29)</f>
         <v>2317.7</v>
       </c>
-      <c r="L11" s="78" t="n">
+      <c r="L11" s="79" t="n">
         <f aca="false">('Balance Sheet'!L6-Drivers!L29)</f>
         <v>3323.80622788275</v>
       </c>
-      <c r="M11" s="78" t="n">
+      <c r="M11" s="79" t="n">
         <f aca="false">('Balance Sheet'!M6-Drivers!M29)</f>
         <v>-8.66885784489568E-007</v>
       </c>
-      <c r="N11" s="78" t="n">
+      <c r="N11" s="79" t="n">
         <f aca="false">('Balance Sheet'!N6-Drivers!N29)</f>
         <v>-4.93056677441928E-006</v>
       </c>
-      <c r="O11" s="78" t="n">
+      <c r="O11" s="79" t="n">
         <f aca="false">('Balance Sheet'!O6-Drivers!O29)</f>
         <v>-2.09666018236021E-005</v>
       </c>
-      <c r="P11" s="78" t="n">
+      <c r="P11" s="79" t="n">
         <f aca="false">('Balance Sheet'!P6-Drivers!P29)</f>
         <v>-6.09262519901677E-005</v>
       </c>
-      <c r="Q11" s="78" t="n">
+      <c r="Q11" s="79" t="n">
         <f aca="false">('Balance Sheet'!Q6-Drivers!Q29)</f>
         <v>2827.89127432764</v>
       </c>
-      <c r="R11" s="78" t="n">
+      <c r="R11" s="79" t="n">
         <f aca="false">('Balance Sheet'!R6-Drivers!R29)</f>
         <v>5924.43110420206</v>
       </c>
-      <c r="S11" s="78" t="n">
+      <c r="S11" s="79" t="n">
         <f aca="false">('Balance Sheet'!S6-Drivers!S29)</f>
         <v>9332.100059432</v>
       </c>
-      <c r="T11" s="78" t="n">
+      <c r="T11" s="79" t="n">
         <f aca="false">('Balance Sheet'!T6-Drivers!T29)</f>
         <v>13072.4148271819</v>
       </c>
-      <c r="U11" s="78" t="n">
+      <c r="U11" s="79" t="n">
         <f aca="false">('Balance Sheet'!U6-Drivers!U29)</f>
         <v>17146.7499330989</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>304</v>
-      </c>
-      <c r="B12" s="78" t="n">
+        <v>316</v>
+      </c>
+      <c r="B12" s="79" t="n">
         <f aca="false">'Balance Sheet'!B18</f>
         <v>0</v>
       </c>
-      <c r="C12" s="78" t="n">
+      <c r="C12" s="79" t="n">
         <f aca="false">'Balance Sheet'!C18</f>
         <v>0</v>
       </c>
-      <c r="D12" s="78" t="n">
+      <c r="D12" s="79" t="n">
         <f aca="false">'Balance Sheet'!D18</f>
         <v>0</v>
       </c>
-      <c r="E12" s="78" t="n">
+      <c r="E12" s="79" t="n">
         <f aca="false">'Balance Sheet'!E18</f>
         <v>0</v>
       </c>
-      <c r="F12" s="78" t="n">
+      <c r="F12" s="79" t="n">
         <f aca="false">'Balance Sheet'!F18</f>
         <v>0</v>
       </c>
-      <c r="G12" s="78" t="n">
+      <c r="G12" s="79" t="n">
         <f aca="false">'Balance Sheet'!G18</f>
         <v>0</v>
       </c>
-      <c r="H12" s="78" t="n">
+      <c r="H12" s="79" t="n">
         <f aca="false">'Balance Sheet'!H18</f>
         <v>0</v>
       </c>
-      <c r="I12" s="78" t="n">
+      <c r="I12" s="79" t="n">
         <f aca="false">'Balance Sheet'!I18</f>
         <v>0</v>
       </c>
-      <c r="J12" s="78" t="n">
+      <c r="J12" s="79" t="n">
         <f aca="false">'Balance Sheet'!J18</f>
         <v>0</v>
       </c>
-      <c r="K12" s="78" t="n">
+      <c r="K12" s="79" t="n">
         <f aca="false">'Balance Sheet'!K18</f>
         <v>0</v>
       </c>
-      <c r="L12" s="78" t="n">
+      <c r="L12" s="79" t="n">
         <f aca="false">'Balance Sheet'!L18</f>
         <v>0</v>
       </c>
-      <c r="M12" s="78" t="n">
+      <c r="M12" s="79" t="n">
         <f aca="false">'Balance Sheet'!M18</f>
         <v>3392.09242260317</v>
       </c>
-      <c r="N12" s="78" t="n">
+      <c r="N12" s="79" t="n">
         <f aca="false">'Balance Sheet'!N18</f>
         <v>4104.81759271949</v>
       </c>
-      <c r="O12" s="78" t="n">
+      <c r="O12" s="79" t="n">
         <f aca="false">'Balance Sheet'!O18</f>
         <v>2535.31698269003</v>
       </c>
-      <c r="P12" s="78" t="n">
+      <c r="P12" s="79" t="n">
         <f aca="false">'Balance Sheet'!P18</f>
         <v>12.1361421654251</v>
       </c>
-      <c r="Q12" s="78" t="n">
+      <c r="Q12" s="79" t="n">
         <f aca="false">'Balance Sheet'!Q18</f>
         <v>0</v>
       </c>
-      <c r="R12" s="78" t="n">
+      <c r="R12" s="79" t="n">
         <f aca="false">'Balance Sheet'!R18</f>
         <v>0</v>
       </c>
-      <c r="S12" s="78" t="n">
+      <c r="S12" s="79" t="n">
         <f aca="false">'Balance Sheet'!S18</f>
         <v>0</v>
       </c>
-      <c r="T12" s="78" t="n">
+      <c r="T12" s="79" t="n">
         <f aca="false">'Balance Sheet'!T18</f>
         <v>0</v>
       </c>
-      <c r="U12" s="78" t="n">
+      <c r="U12" s="79" t="n">
         <f aca="false">'Balance Sheet'!U18</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>305</v>
-      </c>
-      <c r="B13" s="78" t="n">
+        <v>317</v>
+      </c>
+      <c r="B13" s="79" t="n">
         <f aca="false">'Balance Sheet'!B10</f>
         <v>2730.37</v>
       </c>
-      <c r="C13" s="78" t="n">
+      <c r="C13" s="79" t="n">
         <f aca="false">'Balance Sheet'!C10</f>
         <v>3185.89</v>
       </c>
-      <c r="D13" s="78" t="n">
+      <c r="D13" s="79" t="n">
         <f aca="false">'Balance Sheet'!D10</f>
         <v>3256.49</v>
       </c>
-      <c r="E13" s="78" t="n">
+      <c r="E13" s="79" t="n">
         <f aca="false">'Balance Sheet'!E10</f>
         <v>3947.99</v>
       </c>
-      <c r="F13" s="78" t="n">
+      <c r="F13" s="79" t="n">
         <f aca="false">'Balance Sheet'!F10</f>
         <v>4923.98</v>
       </c>
-      <c r="G13" s="78" t="n">
+      <c r="G13" s="79" t="n">
         <f aca="false">'Balance Sheet'!G10</f>
         <v>6133.89</v>
       </c>
-      <c r="H13" s="78" t="n">
+      <c r="H13" s="79" t="n">
         <f aca="false">'Balance Sheet'!H10</f>
         <v>5974.55</v>
       </c>
-      <c r="I13" s="78" t="n">
+      <c r="I13" s="79" t="n">
         <f aca="false">'Balance Sheet'!I10</f>
         <v>7757.46</v>
       </c>
-      <c r="J13" s="78" t="n">
+      <c r="J13" s="79" t="n">
         <f aca="false">'Balance Sheet'!J10</f>
         <v>9522.93</v>
       </c>
-      <c r="K13" s="78" t="n">
+      <c r="K13" s="79" t="n">
         <f aca="false">'Balance Sheet'!K10</f>
         <v>10527.09</v>
       </c>
-      <c r="L13" s="78" t="n">
+      <c r="L13" s="79" t="n">
         <f aca="false">'Balance Sheet'!L10</f>
         <v>17797.87772343</v>
       </c>
-      <c r="M13" s="78" t="n">
+      <c r="M13" s="79" t="n">
         <f aca="false">'Balance Sheet'!M10</f>
         <v>25063.7157652637</v>
       </c>
-      <c r="N13" s="78" t="n">
+      <c r="N13" s="79" t="n">
         <f aca="false">'Balance Sheet'!N10</f>
         <v>26829.0585332768</v>
       </c>
-      <c r="O13" s="78" t="n">
+      <c r="O13" s="79" t="n">
         <f aca="false">'Balance Sheet'!O10</f>
         <v>26970.2814941649</v>
       </c>
-      <c r="P13" s="78" t="n">
+      <c r="P13" s="79" t="n">
         <f aca="false">'Balance Sheet'!P10</f>
         <v>26916.8904837743</v>
       </c>
-      <c r="Q13" s="78" t="n">
+      <c r="Q13" s="79" t="n">
         <f aca="false">'Balance Sheet'!Q10</f>
         <v>27008.5783108577</v>
       </c>
-      <c r="R13" s="78" t="n">
+      <c r="R13" s="79" t="n">
         <f aca="false">'Balance Sheet'!R10</f>
         <v>27271.7298212504</v>
       </c>
-      <c r="S13" s="78" t="n">
+      <c r="S13" s="79" t="n">
         <f aca="false">'Balance Sheet'!S10</f>
         <v>27669.4211544973</v>
       </c>
-      <c r="T13" s="78" t="n">
+      <c r="T13" s="79" t="n">
         <f aca="false">'Balance Sheet'!T10</f>
         <v>28213.4856872016</v>
       </c>
-      <c r="U13" s="78" t="n">
+      <c r="U13" s="79" t="n">
         <f aca="false">'Balance Sheet'!U10</f>
         <v>28886.6293802962</v>
       </c>
@@ -4246,83 +4407,83 @@
       <c r="A14" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="B14" s="78" t="n">
+      <c r="B14" s="79" t="n">
         <f aca="false">Schedules!B24</f>
         <v>1854.23</v>
       </c>
-      <c r="C14" s="78" t="n">
+      <c r="C14" s="79" t="n">
         <f aca="false">Schedules!C24</f>
         <v>2613.07</v>
       </c>
-      <c r="D14" s="78" t="n">
+      <c r="D14" s="79" t="n">
         <f aca="false">Schedules!D24</f>
         <v>2887.67</v>
       </c>
-      <c r="E14" s="78" t="n">
+      <c r="E14" s="79" t="n">
         <f aca="false">Schedules!E24</f>
         <v>2548.22</v>
       </c>
-      <c r="F14" s="78" t="n">
+      <c r="F14" s="79" t="n">
         <f aca="false">Schedules!F24</f>
         <v>2891.17</v>
       </c>
-      <c r="G14" s="78" t="n">
+      <c r="G14" s="79" t="n">
         <f aca="false">Schedules!G24</f>
         <v>3272.12</v>
       </c>
-      <c r="H14" s="78" t="n">
+      <c r="H14" s="79" t="n">
         <f aca="false">Schedules!H24</f>
         <v>3994.62</v>
       </c>
-      <c r="I14" s="78" t="n">
+      <c r="I14" s="79" t="n">
         <f aca="false">Schedules!I24</f>
         <v>8026.36</v>
       </c>
-      <c r="J14" s="78" t="n">
+      <c r="J14" s="79" t="n">
         <f aca="false">Schedules!J24</f>
         <v>9696.9</v>
       </c>
-      <c r="K14" s="78" t="n">
+      <c r="K14" s="79" t="n">
         <f aca="false">Schedules!K24</f>
         <v>10877.5</v>
       </c>
-      <c r="L14" s="78" t="n">
+      <c r="L14" s="79" t="n">
         <f aca="false">Schedules!L24</f>
         <v>18775.8139158579</v>
       </c>
-      <c r="M14" s="78" t="n">
+      <c r="M14" s="79" t="n">
         <f aca="false">Schedules!M24</f>
         <v>20841.5636505861</v>
       </c>
-      <c r="N14" s="78" t="n">
+      <c r="N14" s="79" t="n">
         <f aca="false">Schedules!N24</f>
         <v>22981.2544470552</v>
       </c>
-      <c r="O14" s="78" t="n">
+      <c r="O14" s="79" t="n">
         <f aca="false">Schedules!O24</f>
         <v>25583.3586191545</v>
       </c>
-      <c r="P14" s="78" t="n">
+      <c r="P14" s="79" t="n">
         <f aca="false">Schedules!P24</f>
         <v>28604.4102080769</v>
       </c>
-      <c r="Q14" s="78" t="n">
+      <c r="Q14" s="79" t="n">
         <f aca="false">Schedules!Q24</f>
         <v>32076.4813411262</v>
       </c>
-      <c r="R14" s="78" t="n">
+      <c r="R14" s="79" t="n">
         <f aca="false">Schedules!R24</f>
         <v>35985.8605122595</v>
       </c>
-      <c r="S14" s="78" t="n">
+      <c r="S14" s="79" t="n">
         <f aca="false">Schedules!S24</f>
         <v>40352.9630083805</v>
       </c>
-      <c r="T14" s="78" t="n">
+      <c r="T14" s="79" t="n">
         <f aca="false">Schedules!T24</f>
         <v>45199.3889170401</v>
       </c>
-      <c r="U14" s="78" t="n">
+      <c r="U14" s="79" t="n">
         <f aca="false">Schedules!U24</f>
         <v>50538.4554344112</v>
       </c>
@@ -6666,11 +6827,11 @@
         <v>0.5</v>
       </c>
       <c r="C43" s="36" t="n">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="D43" s="37" t="n">
         <f aca="false">B43*C43</f>
-        <v>64.5</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6682,11 +6843,11 @@
         <v>0.25</v>
       </c>
       <c r="C44" s="36" t="n">
-        <v>155</v>
+        <v>129</v>
       </c>
       <c r="D44" s="37" t="n">
         <f aca="false">B44*C44</f>
-        <v>38.75</v>
+        <v>32.25</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6698,11 +6859,11 @@
         <v>0.25</v>
       </c>
       <c r="C45" s="36" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D45" s="37" t="n">
         <f aca="false">B45*C45</f>
-        <v>15</v>
+        <v>14.5</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6715,7 +6876,7 @@
       </c>
       <c r="D46" s="38" t="n">
         <f aca="false">SUM(D43:D45)</f>
-        <v>118.25</v>
+        <v>107.25</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6723,8 +6884,8 @@
         <v>127</v>
       </c>
       <c r="B48" s="39" t="n">
-        <f aca="false">DCF!B33</f>
-        <v>129.40298338516</v>
+        <f aca="false">DCF!B43</f>
+        <v>121.083756994038</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6733,7 +6894,7 @@
       </c>
       <c r="B49" s="37" t="n">
         <f aca="false">INDEX(C43:C45,Scenarios!$B$4)</f>
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>